<commit_message>
Atualiza regras de insumos e ajustes do pipeline de setembro
</commit_message>
<xml_diff>
--- a/utils/insumos/regra_ajuste_final.xlsx
+++ b/utils/insumos/regra_ajuste_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hapvida-my.sharepoint.com/personal/anderson_dossantos_hapvida_com_br/Documents/5 Estrelas/INSUMOS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anderson.dossantos\Desktop\dev\5 Estrelas\utils\insumos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_EC45D2F3D3E7DFA4EEC3AE370F8F7C5523BAC60A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA6B2EF7-BC43-4DAE-A867-DE406AD8FC97}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52FCC33F-2031-4475-A2D9-90DF222659C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="regras_ajuste_final" sheetId="1" r:id="rId1"/>
@@ -19,14 +19,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">comparadores!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">regras_ajuste_final!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">regras_ajuste_final!$A$1:$P$17</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="119">
   <si>
     <t>STATUS_ATIVO</t>
   </si>
@@ -112,70 +112,127 @@
     <t>Ajusta Notre Dame SP para Hospital Sao Lucas</t>
   </si>
   <si>
+    <t>CLASSIFICACAO</t>
+  </si>
+  <si>
+    <t>MED PREV</t>
+  </si>
+  <si>
+    <t>NASCER BEM</t>
+  </si>
+  <si>
+    <t>ESPECIALIDADE</t>
+  </si>
+  <si>
+    <t>PLANEJAMENTO FAMILIAR- NB</t>
+  </si>
+  <si>
+    <t>MEDICINA PREVENTIVA BOA VISTA</t>
+  </si>
+  <si>
+    <t>valores indevidamente indo para nascer bem</t>
+  </si>
+  <si>
+    <t>QUALIVIDA</t>
+  </si>
+  <si>
+    <t>nao</t>
+  </si>
+  <si>
+    <t>OBSTETRICIA ALTO RISCO</t>
+  </si>
+  <si>
+    <t>CLINICA E DIAG ZONA LESTE</t>
+  </si>
+  <si>
+    <t>INATIVA: obstetricia alto risco em CLINICA E DIAG ZONA LESTE deve permanecer como NASCER BEM. A regra anterior sobrescrevia NASCER BEM para MED PREV no ajuste final.</t>
+  </si>
+  <si>
+    <t>HOSPITAL MATERNIDADE RP</t>
+  </si>
+  <si>
+    <t>INATIVA: obstetricia alto risco em HOSPITAL MATERNIDADE RP deve permanecer como NASCER BEM. A regra anterior sobrescrevia NASCER BEM para MED PREV no ajuste final.</t>
+  </si>
+  <si>
+    <t>HOSPITAL ARARAQUARA</t>
+  </si>
+  <si>
+    <t>INATIVA: obstetricia alto risco em HOSPITAL ARARAQUARA deve permanecer como NASCER BEM. A regra anterior sobrescrevia NASCER BEM para MED PREV no ajuste final.</t>
+  </si>
+  <si>
+    <t>PROCEDIMENTO</t>
+  </si>
+  <si>
+    <t>EXAME ANATOMO PATOLOGICO POR ORGAO BIOPSIA OU BIOPSIA ASPIRATIVA</t>
+  </si>
+  <si>
+    <t>COLUNA:PROFISSIONAL</t>
+  </si>
+  <si>
+    <t>ODONTOLOGIA</t>
+  </si>
+  <si>
+    <t>vazio</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Para odontologia sem local, usa profissional como local editado</t>
+  </si>
+  <si>
+    <t>CONTRATACAO</t>
+  </si>
+  <si>
+    <t>rede credenciada</t>
+  </si>
+  <si>
+    <t>HAPVIDA ASSISTENCIA MEDICA S.A</t>
+  </si>
+  <si>
+    <t>HAPCLINICA</t>
+  </si>
+  <si>
+    <t>TIPO</t>
+  </si>
+  <si>
+    <t>CLINICA ITUPEVA</t>
+  </si>
+  <si>
+    <t>um medico especifico atende por rede propria em clinica credenciada</t>
+  </si>
+  <si>
+    <t>rede propria</t>
+  </si>
+  <si>
+    <t>AMBULANCIA; AMBULÂNCIA</t>
+  </si>
+  <si>
+    <t>colocando todas as ambulancias para rede propria</t>
+  </si>
+  <si>
     <t>excluir</t>
   </si>
   <si>
-    <t>CLASSIFICACAO</t>
-  </si>
-  <si>
-    <t>AMBULÂNCIA</t>
-  </si>
-  <si>
-    <t>Exclui classificacao ambulancia</t>
-  </si>
-  <si>
-    <t>MED PREV</t>
-  </si>
-  <si>
-    <t>NASCER BEM</t>
-  </si>
-  <si>
-    <t>ESPECIALIDADE</t>
-  </si>
-  <si>
-    <t>PLANEJAMENTO FAMILIAR- NB</t>
-  </si>
-  <si>
-    <t>MEDICINA PREVENTIVA BOA VISTA</t>
-  </si>
-  <si>
-    <t>valores indevidamente indo para nascer bem</t>
-  </si>
-  <si>
-    <t>QUALIVIDA</t>
-  </si>
-  <si>
-    <t>OBSTETRICIA ALTO RISCO</t>
-  </si>
-  <si>
-    <t>CLINICA E DIAG ZONA LESTE</t>
-  </si>
-  <si>
-    <t>HOSPITAL MATERNIDADE RP</t>
-  </si>
-  <si>
-    <t>HOSPITAL ARARAQUARA</t>
-  </si>
-  <si>
-    <t>PROCEDIMENTO</t>
-  </si>
-  <si>
-    <t>EXAME ANATOMO PATOLOGICO POR ORGAO BIOPSIA OU BIOPSIA ASPIRATIVA</t>
-  </si>
-  <si>
-    <t>COLUNA:PROFISSIONAL</t>
-  </si>
-  <si>
-    <t>ODONTOLOGIA</t>
-  </si>
-  <si>
-    <t>vazio</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Para odontologia sem local, usa profissional como local editado</t>
+    <t>Exclui todas as linhas classificadas como ambulancia</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>Exclui linhas com TIPO 15</t>
+  </si>
+  <si>
+    <t>TELECONSULTA CASE</t>
+  </si>
+  <si>
+    <t>contem</t>
+  </si>
+  <si>
+    <t>PGC</t>
+  </si>
+  <si>
+    <t>Ajuste criado porque alguns atendimentos PGC chegam com TIPO 4 por erro de origem, ficam fora da regra principal de TELECONSULTA CASE e caem em MED PREV.</t>
   </si>
   <si>
     <t>COMPARADOR</t>
@@ -199,9 +256,6 @@
     <t>Valor da coluna nao deve estar em lista separada por ponto e virgula.</t>
   </si>
   <si>
-    <t>contem</t>
-  </si>
-  <si>
     <t>Texto da coluna deve conter o valor informado.</t>
   </si>
   <si>
@@ -280,9 +334,6 @@
     <t>CE</t>
   </si>
   <si>
-    <t>nao</t>
-  </si>
-  <si>
     <t>HOSPITAL ANA LIMA</t>
   </si>
   <si>
@@ -292,9 +343,6 @@
     <t>Objetivo: quando CLASSIFICACAO = ODONTOLOGIA, TIPO = 5 e LOCAL EDITADO estiver vazio, preencher LOCAL EDITADO com PROFISSIONAL.</t>
   </si>
   <si>
-    <t>TIPO</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
@@ -316,20 +364,32 @@
     <t>ACAO = excluir, COLUNA_FILTRO_1 = CLASSIFICACAO, COMPARADOR_1 = igual, VALOR_1 = AMBULANCIA.</t>
   </si>
   <si>
-    <t>HAPVIDA ASSISTENCIA MEDICA S.A</t>
-  </si>
-  <si>
-    <t>CONTRATACAO</t>
-  </si>
-  <si>
-    <t>rede credenciada</t>
+    <t xml:space="preserve">sim </t>
+  </si>
+  <si>
+    <t>MED PREV HORTO FLORESTAL</t>
+  </si>
+  <si>
+    <t>ajuste criado pois med prev está caindo em como TIPO 2</t>
+  </si>
+  <si>
+    <t>MED PREV CACHOEIRINHA</t>
+  </si>
+  <si>
+    <t>NOME UNIDADE</t>
+  </si>
+  <si>
+    <t>ESPECIALIDADE  TESTE</t>
+  </si>
+  <si>
+    <t>exclusão cirada pq aparentemente a linha foi criada como teste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -356,6 +416,12 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -385,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -397,6 +463,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Excel Built-in Title" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -662,7 +729,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -781,27 +848,57 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" ht="15" customHeight="1">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3" t="s">
         <v>25</v>
       </c>
       <c r="J3" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" t="s">
+        <v>33</v>
+      </c>
+      <c r="N3" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" t="s">
         <v>30</v>
       </c>
       <c r="Q3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1">
@@ -809,31 +906,31 @@
         <v>17</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
       </c>
       <c r="D4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" t="s">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
         <v>32</v>
-      </c>
-      <c r="F4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>35</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>21</v>
@@ -842,19 +939,19 @@
         <v>25</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O4" t="s">
         <v>25</v>
       </c>
       <c r="P4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q4" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1">
@@ -862,31 +959,31 @@
         <v>17</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
-        <v>32</v>
-      </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
         <v>17</v>
       </c>
       <c r="H5" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I5" t="s">
         <v>25</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>21</v>
@@ -898,16 +995,16 @@
         <v>38</v>
       </c>
       <c r="N5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O5" t="s">
         <v>25</v>
       </c>
       <c r="P5" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="Q5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15" customHeight="1">
@@ -915,31 +1012,31 @@
         <v>17</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s">
         <v>29</v>
       </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G6" t="s">
         <v>17</v>
       </c>
       <c r="H6" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I6" t="s">
         <v>25</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>21</v>
@@ -951,16 +1048,16 @@
         <v>40</v>
       </c>
       <c r="N6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O6" t="s">
         <v>25</v>
       </c>
       <c r="P6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Q6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1">
@@ -968,31 +1065,31 @@
         <v>17</v>
       </c>
       <c r="B7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
         <v>18</v>
       </c>
       <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
         <v>29</v>
       </c>
-      <c r="E7" t="s">
-        <v>32</v>
-      </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G7" t="s">
         <v>17</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="I7" t="s">
         <v>25</v>
       </c>
       <c r="J7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>21</v>
@@ -1001,19 +1098,19 @@
         <v>25</v>
       </c>
       <c r="M7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O7" t="s">
         <v>25</v>
       </c>
       <c r="P7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="Q7" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1">
@@ -1021,152 +1118,137 @@
         <v>17</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
         <v>18</v>
       </c>
       <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
         <v>29</v>
       </c>
-      <c r="E8" t="s">
-        <v>32</v>
-      </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
       </c>
       <c r="H8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L8" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" t="s">
+        <v>25</v>
+      </c>
+      <c r="P8" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q8" t="s">
         <v>34</v>
       </c>
-      <c r="I8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J8" t="s">
-        <v>39</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8" t="s">
-        <v>25</v>
-      </c>
-      <c r="M8" t="s">
-        <v>42</v>
-      </c>
-      <c r="N8" t="s">
-        <v>29</v>
-      </c>
-      <c r="O8" t="s">
-        <v>25</v>
-      </c>
-      <c r="P8" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" ht="15" customHeight="1">
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" t="s">
         <v>17</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="H9" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="I9" t="s">
         <v>25</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="L9" t="s">
-        <v>25</v>
-      </c>
-      <c r="M9" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="N9" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="O9" t="s">
         <v>25</v>
       </c>
       <c r="P9" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="Q9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="15" customHeight="1">
       <c r="A10" t="s">
         <v>17</v>
       </c>
       <c r="B10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" t="s">
-        <v>45</v>
+        <v>51</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="H10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I10" t="s">
         <v>25</v>
       </c>
       <c r="J10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K10" t="s">
         <v>19</v>
       </c>
       <c r="L10" t="s">
-        <v>47</v>
-      </c>
-      <c r="N10" t="s">
-        <v>21</v>
-      </c>
-      <c r="O10" t="s">
-        <v>25</v>
-      </c>
-      <c r="P10" t="s">
-        <v>48</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>49</v>
+        <v>25</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1">
@@ -1174,37 +1256,37 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" t="s">
         <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="H11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I11" t="s">
         <v>25</v>
       </c>
       <c r="J11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="L11" t="s">
         <v>25</v>
       </c>
-      <c r="M11" s="4" t="s">
-        <v>96</v>
+      <c r="M11" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="15" customHeight="1">
@@ -1212,43 +1294,282 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>97</v>
+        <v>28</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>98</v>
+        <v>54</v>
       </c>
       <c r="G12" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="H12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I12" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12">
+        <v>2</v>
+      </c>
+      <c r="K12" t="s">
+        <v>19</v>
+      </c>
+      <c r="L12" t="s">
+        <v>25</v>
+      </c>
+      <c r="M12" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="15" customHeight="1">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J14" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17">
+      <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" t="s">
+        <v>55</v>
+      </c>
+      <c r="I15" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>65</v>
+      </c>
+      <c r="F16" t="s">
         <v>29</v>
       </c>
-      <c r="I12" t="s">
-        <v>25</v>
-      </c>
-      <c r="J12" t="s">
-        <v>46</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>31</v>
+      </c>
+      <c r="I16" t="s">
+        <v>66</v>
+      </c>
+      <c r="J16" t="s">
+        <v>67</v>
+      </c>
+      <c r="K16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L16" t="s">
+        <v>25</v>
+      </c>
+      <c r="M16">
+        <v>4</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="15" customHeight="1">
+      <c r="A17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G17" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" t="s">
+        <v>55</v>
+      </c>
+      <c r="I17" t="s">
+        <v>25</v>
+      </c>
+      <c r="J17">
+        <v>2</v>
+      </c>
+      <c r="K17" t="s">
+        <v>19</v>
+      </c>
+      <c r="L17" t="s">
+        <v>25</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="15" customHeight="1">
+      <c r="A18" t="s">
+        <v>112</v>
+      </c>
+      <c r="B18">
+        <v>18</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" t="s">
+        <v>36</v>
+      </c>
+      <c r="H18" t="s">
+        <v>55</v>
+      </c>
+      <c r="I18" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="K18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18" t="s">
+        <v>25</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="15" customHeight="1">
+      <c r="A19" t="s">
+        <v>112</v>
+      </c>
+      <c r="B19">
+        <v>19</v>
+      </c>
+      <c r="C19" t="s">
+        <v>61</v>
+      </c>
+      <c r="H19" t="s">
         <v>21</v>
       </c>
-      <c r="L12" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" t="s">
-        <v>48</v>
+      <c r="I19" t="s">
+        <v>25</v>
+      </c>
+      <c r="J19" t="s">
+        <v>116</v>
+      </c>
+      <c r="K19" t="s">
+        <v>31</v>
+      </c>
+      <c r="L19" t="s">
+        <v>25</v>
+      </c>
+      <c r="M19" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:P17" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555596" footer="0.51180555555555596"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Aptos,Regular"&amp;1 &amp;Kff0000 INTERNO#_x000D_</oddHeader>
     <oddFooter>&amp;C&amp;"Aptos,Regular"&amp;10 &amp;Kff0000_x000D_# INTERNO</oddFooter>
@@ -1267,7 +1588,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>16</v>
@@ -1278,15 +1599,15 @@
         <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
@@ -1294,47 +1615,47 @@
         <v>22</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1359,23 +1680,23 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21.75" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="B1" s="3"/>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15" customHeight="1">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15" customHeight="1">
@@ -1383,7 +1704,7 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15" customHeight="1">
@@ -1391,7 +1712,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15" customHeight="1">
@@ -1399,7 +1720,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15" customHeight="1">
@@ -1407,7 +1728,7 @@
         <v>4</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" customHeight="1">
@@ -1415,7 +1736,7 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="15" customHeight="1">
@@ -1423,31 +1744,31 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15" customHeight="1">
       <c r="A13" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="B13" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="15" customHeight="1">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15" customHeight="1">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="15" customHeight="1">
@@ -1455,17 +1776,17 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
@@ -1481,7 +1802,7 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
@@ -1489,7 +1810,7 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1">
@@ -1513,17 +1834,17 @@
         <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15" customHeight="1">
       <c r="A27" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15" customHeight="1">
       <c r="A28" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
@@ -1539,7 +1860,7 @@
         <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15" customHeight="1">
@@ -1547,7 +1868,7 @@
         <v>6</v>
       </c>
       <c r="B31" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="15" customHeight="1">
@@ -1555,7 +1876,7 @@
         <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15" customHeight="1">
@@ -1571,7 +1892,7 @@
         <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="15" customHeight="1">
@@ -1579,7 +1900,7 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>88</v>
+        <v>55</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="15" customHeight="1">
@@ -1595,7 +1916,7 @@
         <v>12</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="15" customHeight="1">
@@ -1611,22 +1932,22 @@
         <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="15" customHeight="1">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15" customHeight="1">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="15" customHeight="1">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:2">
@@ -1634,15 +1955,15 @@
         <v>2</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>